<commit_message>
made adjustments to GUI and ICSW process
</commit_message>
<xml_diff>
--- a/app/templates/product_input_template.xlsx
+++ b/app/templates/product_input_template.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -435,16 +435,15 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,55 +474,50 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>BASE PRICE</t>
+          <t>LIST PRICE</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>LIST PRICE</t>
+          <t>LENGTH</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>WIDTH</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>WIDTH</t>
+          <t>HEIGHT</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>HEIGHT</t>
+          <t>WEIGHT</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>BRAND CODE</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>BRAND CODE</t>
+          <t>PRODUCT CAT</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>PRODUCT CAT</t>
+          <t>WEBSITE CAT</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>WEBSITE CAT</t>
+          <t>PRODLINE</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>PRODLINE</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>SEASONAL</t>
         </is>
@@ -548,10 +542,10 @@
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
@@ -562,30 +556,27 @@
       <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>BRANDX</t>
+        </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>BRANDX</t>
+          <t>CATEG1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>CATEG1</t>
+          <t>WEBCAT1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>WEBCAT1</t>
+          <t>LINE1</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
-        <is>
-          <t>LINE1</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
         <is>
           <t>n</t>
         </is>
@@ -602,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -715,7 +706,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BASE PRICE</t>
+          <t>LIST PRICE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -725,14 +716,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Optional: Override calculated base price</t>
+          <t>Optional: Override calculated list price</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LIST PRICE</t>
+          <t>SEASONAL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -741,23 +732,6 @@
         </is>
       </c>
       <c r="C8" t="inlineStr">
-        <is>
-          <t>Optional: Override calculated list price</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SEASONAL</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
         <is>
           <t>Enter y for seasonal products, n for standard</t>
         </is>

</xml_diff>